<commit_message>
commit 12 April 2026
</commit_message>
<xml_diff>
--- a/axis-remit-automation/src/test/resources/testdata/TestData.xlsx
+++ b/axis-remit-automation/src/test/resources/testdata/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7620"/>
+    <workbookView windowWidth="19635" windowHeight="7020"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
   <si>
     <t>baseUrl</t>
   </si>
@@ -1317,9 +1317,7 @@
       <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
         <v>11</v>
       </c>

</xml_diff>